<commit_message>
test DPE correct harmonized dataset colum
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NHATS.xlsx
+++ b/baseline/data_processing_elements-NHATS.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17bc974f5891b333/Documents/ProPASS/Harmo/NHATS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\riconf\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="443" documentId="8_{9B09118A-A407-4BA8-95FA-BC26F1D8B61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABBF837A-2B70-46A1-A86C-7E16F6AB2487}"/>
   <bookViews>
-    <workbookView xWindow="71880" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F744FAC3-0BAB-4C7A-92B3-0824573F48DB}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8688"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Y$166</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="400">
   <si>
     <t>index</t>
   </si>
@@ -1622,8 +1621,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1785,8 +1784,8 @@
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{046646FB-A022-4AA6-8EBD-3A31D1B63504}"/>
-    <cellStyle name="Normal 3" xfId="1" xr:uid="{7D2CC4ED-5DE6-422B-B2D7-BFBF631E5EC7}"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 3" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2117,36 +2116,36 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC73F24-28B6-451D-9DE2-0CD6B57BA63C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z164"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="9.1328125" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
     <col min="2" max="2" width="24.33203125" customWidth="1"/>
-    <col min="3" max="3" width="31.9296875" customWidth="1"/>
-    <col min="4" max="4" width="37.1328125" customWidth="1"/>
-    <col min="5" max="5" width="22.3984375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.1328125" customWidth="1"/>
-    <col min="8" max="8" width="15.265625" customWidth="1"/>
+    <col min="3" max="3" width="31.94921875" customWidth="1"/>
+    <col min="4" max="4" width="37.140625" customWidth="1"/>
+    <col min="5" max="5" width="22.37890625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" customWidth="1"/>
     <col min="9" max="11" width="25.33203125" customWidth="1"/>
-    <col min="12" max="12" width="29.9296875" customWidth="1"/>
-    <col min="13" max="13" width="57.3984375" style="2" customWidth="1"/>
-    <col min="14" max="14" width="70.3984375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="22.1328125" customWidth="1"/>
-    <col min="16" max="16" width="22.1328125" style="11" customWidth="1"/>
-    <col min="17" max="17" width="22.1328125" style="12" customWidth="1"/>
-    <col min="18" max="18" width="24.53125" style="13" customWidth="1"/>
-    <col min="19" max="19" width="22.1328125" style="15" customWidth="1"/>
-    <col min="20" max="20" width="31.86328125" style="16" customWidth="1"/>
-    <col min="21" max="21" width="21.1328125" customWidth="1"/>
-    <col min="22" max="22" width="28.46484375" customWidth="1"/>
-    <col min="23" max="23" width="23.73046875" customWidth="1"/>
+    <col min="12" max="12" width="29.94921875" customWidth="1"/>
+    <col min="13" max="13" width="57.37890625" style="2" customWidth="1"/>
+    <col min="14" max="14" width="70.37890625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="22.140625" customWidth="1"/>
+    <col min="16" max="16" width="22.140625" style="11" customWidth="1"/>
+    <col min="17" max="17" width="22.140625" style="12" customWidth="1"/>
+    <col min="18" max="18" width="24.5234375" style="13" customWidth="1"/>
+    <col min="19" max="19" width="22.140625" style="15" customWidth="1"/>
+    <col min="20" max="20" width="31.85546875" style="16" customWidth="1"/>
+    <col min="21" max="21" width="21.140625" customWidth="1"/>
+    <col min="22" max="22" width="28.47265625" customWidth="1"/>
+    <col min="23" max="23" width="23.7109375" customWidth="1"/>
     <col min="24" max="24" width="27.6640625" customWidth="1"/>
-    <col min="25" max="25" width="61.59765625" customWidth="1"/>
-    <col min="26" max="26" width="22.46484375" customWidth="1"/>
+    <col min="25" max="25" width="61.6171875" customWidth="1"/>
+    <col min="26" max="26" width="22.47265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:26" s="1" customFormat="1" ht="15.75">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -2226,9 +2225,12 @@
         <v>399</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:26" ht="15.75">
       <c r="A2">
         <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>294</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -2280,9 +2282,12 @@
       </c>
       <c r="Z2" s="4"/>
     </row>
-    <row r="3" spans="1:26" s="21" customFormat="1" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:26" s="21" customFormat="1" ht="42.75">
       <c r="A3" s="18">
         <v>2</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>294</v>
       </c>
       <c r="C3" s="21" t="s">
         <v>20</v>
@@ -2336,9 +2341,12 @@
       </c>
       <c r="Z3" s="24"/>
     </row>
-    <row r="4" spans="1:26" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:26" ht="85.5">
       <c r="A4" s="18">
         <v>3</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>294</v>
       </c>
       <c r="C4" t="s">
         <v>25</v>
@@ -2392,9 +2400,12 @@
       </c>
       <c r="Z4" s="18"/>
     </row>
-    <row r="5" spans="1:26" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:26" ht="42.75">
       <c r="A5" s="18">
         <v>4</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>294</v>
       </c>
       <c r="C5" t="s">
         <v>32</v>
@@ -2448,10 +2459,13 @@
       </c>
       <c r="Z5" s="18"/>
     </row>
-    <row r="6" spans="1:26" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:26" ht="99.75">
       <c r="A6" s="18">
         <v>5</v>
       </c>
+      <c r="B6" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C6" t="s">
         <v>36</v>
       </c>
@@ -2500,10 +2514,13 @@
         <v>303</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:26" ht="151.80000000000001">
       <c r="A7" s="18">
         <v>6</v>
       </c>
+      <c r="B7" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C7" t="s">
         <v>279</v>
       </c>
@@ -2554,10 +2571,13 @@
         <v>309</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:26" ht="28.5">
       <c r="A8" s="18">
         <v>7</v>
       </c>
+      <c r="B8" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C8" t="s">
         <v>42</v>
       </c>
@@ -2608,10 +2628,13 @@
       </c>
       <c r="Z8" s="18"/>
     </row>
-    <row r="9" spans="1:26" s="21" customFormat="1" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:26" s="21" customFormat="1" ht="96.6">
       <c r="A9" s="18">
         <v>8</v>
       </c>
+      <c r="B9" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C9" s="21" t="s">
         <v>46</v>
       </c>
@@ -2661,10 +2684,13 @@
         <v>391</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:26" ht="27.6">
       <c r="A10" s="18">
         <v>9</v>
       </c>
+      <c r="B10" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C10" t="s">
         <v>50</v>
       </c>
@@ -2712,10 +2738,13 @@
       </c>
       <c r="Z10" s="18"/>
     </row>
-    <row r="11" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:26" ht="27.6">
       <c r="A11" s="18">
         <v>10</v>
       </c>
+      <c r="B11" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C11" t="s">
         <v>55</v>
       </c>
@@ -2757,10 +2786,13 @@
       </c>
       <c r="Z11" s="18"/>
     </row>
-    <row r="12" spans="1:26" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:26" ht="41.4">
       <c r="A12" s="18">
         <v>11</v>
       </c>
+      <c r="B12" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C12" t="s">
         <v>58</v>
       </c>
@@ -2811,11 +2843,13 @@
       </c>
       <c r="Z12" s="18"/>
     </row>
-    <row r="13" spans="1:26" ht="171" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:26" ht="165.6">
       <c r="A13" s="18">
         <v>12</v>
       </c>
-      <c r="B13" s="21"/>
+      <c r="B13" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C13" s="21" t="s">
         <v>62</v>
       </c>
@@ -2875,10 +2909,13 @@
         <v>323</v>
       </c>
     </row>
-    <row r="14" spans="1:26" ht="171" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:26" ht="165.6">
       <c r="A14" s="18">
         <v>13</v>
       </c>
+      <c r="B14" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C14" t="s">
         <v>66</v>
       </c>
@@ -2929,10 +2966,13 @@
       </c>
       <c r="Z14" s="18"/>
     </row>
-    <row r="15" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:26" ht="27.6">
       <c r="A15" s="18">
         <v>14</v>
       </c>
+      <c r="B15" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C15" t="s">
         <v>70</v>
       </c>
@@ -2977,10 +3017,13 @@
       </c>
       <c r="Z15" s="18"/>
     </row>
-    <row r="16" spans="1:26" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:26" ht="124.2">
       <c r="A16" s="18">
         <v>15</v>
       </c>
+      <c r="B16" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C16" t="s">
         <v>73</v>
       </c>
@@ -3035,10 +3078,13 @@
       </c>
       <c r="Z16" s="18"/>
     </row>
-    <row r="17" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:26" ht="27.6">
       <c r="A17" s="18">
         <v>16</v>
       </c>
+      <c r="B17" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C17" t="s">
         <v>79</v>
       </c>
@@ -3083,9 +3129,12 @@
       </c>
       <c r="Z17" s="18"/>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:26">
       <c r="A18" s="18">
         <v>17</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>294</v>
       </c>
       <c r="C18" t="s">
         <v>82</v>
@@ -3138,9 +3187,12 @@
       </c>
       <c r="Z18" s="18"/>
     </row>
-    <row r="19" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:26" ht="27.6">
       <c r="A19" s="18">
         <v>18</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>294</v>
       </c>
       <c r="C19" t="s">
         <v>86</v>
@@ -3191,10 +3243,13 @@
       </c>
       <c r="Z19" s="18"/>
     </row>
-    <row r="20" spans="1:26" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:26" ht="179.4">
       <c r="A20" s="18">
         <v>19</v>
       </c>
+      <c r="B20" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C20" t="s">
         <v>88</v>
       </c>
@@ -3245,10 +3300,13 @@
       </c>
       <c r="Z20" s="18"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:26">
       <c r="A21" s="18">
         <v>20</v>
       </c>
+      <c r="B21" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C21" t="s">
         <v>91</v>
       </c>
@@ -3300,10 +3358,13 @@
       </c>
       <c r="Z21" s="18"/>
     </row>
-    <row r="22" spans="1:26" ht="57" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:26" ht="55.2">
       <c r="A22" s="18">
         <v>21</v>
       </c>
+      <c r="B22" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C22" t="s">
         <v>93</v>
       </c>
@@ -3354,10 +3415,13 @@
       </c>
       <c r="Z22" s="18"/>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:26">
       <c r="A23" s="18">
         <v>22</v>
       </c>
+      <c r="B23" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C23" t="s">
         <v>95</v>
       </c>
@@ -3390,10 +3454,13 @@
       </c>
       <c r="Z23" s="18"/>
     </row>
-    <row r="24" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:26" ht="27.6">
       <c r="A24" s="18">
         <v>23</v>
       </c>
+      <c r="B24" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C24" t="s">
         <v>98</v>
       </c>
@@ -3435,10 +3502,13 @@
       </c>
       <c r="Z24" s="18"/>
     </row>
-    <row r="25" spans="1:26" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:26" ht="41.4">
       <c r="A25" s="18">
         <v>24</v>
       </c>
+      <c r="B25" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C25" t="s">
         <v>100</v>
       </c>
@@ -3483,10 +3553,13 @@
       </c>
       <c r="Z25" s="18"/>
     </row>
-    <row r="26" spans="1:26" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:26" ht="41.4">
       <c r="A26" s="18">
         <v>25</v>
       </c>
+      <c r="B26" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C26" t="s">
         <v>104</v>
       </c>
@@ -3531,10 +3604,13 @@
       </c>
       <c r="Z26" s="18"/>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:26">
       <c r="A27" s="18">
         <v>26</v>
       </c>
+      <c r="B27" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C27" t="s">
         <v>107</v>
       </c>
@@ -3579,10 +3655,13 @@
       </c>
       <c r="Z27" s="18"/>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:26">
       <c r="A28" s="18">
         <v>27</v>
       </c>
+      <c r="B28" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C28" t="s">
         <v>110</v>
       </c>
@@ -3628,10 +3707,13 @@
       </c>
       <c r="Z28" s="18"/>
     </row>
-    <row r="29" spans="1:26" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:26" ht="41.4">
       <c r="A29" s="18">
         <v>28</v>
       </c>
+      <c r="B29" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C29" t="s">
         <v>113</v>
       </c>
@@ -3676,10 +3758,13 @@
       </c>
       <c r="Z29" s="18"/>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:26">
       <c r="A30" s="18">
         <v>29</v>
       </c>
+      <c r="B30" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C30" t="s">
         <v>116</v>
       </c>
@@ -3724,10 +3809,13 @@
       </c>
       <c r="Z30" s="18"/>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:26">
       <c r="A31" s="18">
         <v>30</v>
       </c>
+      <c r="B31" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C31" t="s">
         <v>119</v>
       </c>
@@ -3772,10 +3860,13 @@
       </c>
       <c r="Z31" s="18"/>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:26">
       <c r="A32" s="18">
         <v>31</v>
       </c>
+      <c r="B32" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C32" t="s">
         <v>122</v>
       </c>
@@ -3820,10 +3911,13 @@
       </c>
       <c r="Z32" s="18"/>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:26">
       <c r="A33" s="18">
         <v>32</v>
       </c>
+      <c r="B33" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C33" t="s">
         <v>125</v>
       </c>
@@ -3868,10 +3962,13 @@
       </c>
       <c r="Z33" s="18"/>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:26">
       <c r="A34" s="18">
         <v>33</v>
       </c>
+      <c r="B34" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C34" t="s">
         <v>127</v>
       </c>
@@ -3916,10 +4013,13 @@
       </c>
       <c r="Z34" s="18"/>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:26">
       <c r="A35" s="18">
         <v>34</v>
       </c>
+      <c r="B35" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C35" t="s">
         <v>129</v>
       </c>
@@ -3964,10 +4064,13 @@
       </c>
       <c r="Z35" s="18"/>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:26">
       <c r="A36" s="18">
         <v>35</v>
       </c>
+      <c r="B36" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C36" t="s">
         <v>131</v>
       </c>
@@ -4012,10 +4115,13 @@
       </c>
       <c r="Z36" s="18"/>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:26">
       <c r="A37" s="18">
         <v>36</v>
       </c>
+      <c r="B37" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C37" t="s">
         <v>133</v>
       </c>
@@ -4060,10 +4166,13 @@
       </c>
       <c r="Z37" s="18"/>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:26">
       <c r="A38" s="18">
         <v>37</v>
       </c>
+      <c r="B38" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C38" t="s">
         <v>136</v>
       </c>
@@ -4109,11 +4218,13 @@
       </c>
       <c r="Z38" s="18"/>
     </row>
-    <row r="39" spans="1:26" s="2" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:26" s="2" customFormat="1" ht="46.5" customHeight="1">
       <c r="A39" s="18">
         <v>38</v>
       </c>
-      <c r="B39"/>
+      <c r="B39" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C39" s="2" t="s">
         <v>140</v>
       </c>
@@ -4162,10 +4273,13 @@
         <v>17</v>
       </c>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:26">
       <c r="A40" s="18">
         <v>39</v>
       </c>
+      <c r="B40" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C40" t="s">
         <v>144</v>
       </c>
@@ -4211,10 +4325,13 @@
       </c>
       <c r="Z40" s="18"/>
     </row>
-    <row r="41" spans="1:26" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:26" ht="41.4">
       <c r="A41" s="18">
         <v>40</v>
       </c>
+      <c r="B41" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C41" t="s">
         <v>147</v>
       </c>
@@ -4259,10 +4376,13 @@
       </c>
       <c r="Z41" s="18"/>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:26">
       <c r="A42" s="18">
         <v>41</v>
       </c>
+      <c r="B42" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C42" t="s">
         <v>150</v>
       </c>
@@ -4307,10 +4427,13 @@
       </c>
       <c r="Z42" s="18"/>
     </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:26">
       <c r="A43" s="18">
         <v>42</v>
       </c>
+      <c r="B43" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C43" t="s">
         <v>153</v>
       </c>
@@ -4356,10 +4479,13 @@
       </c>
       <c r="Z43" s="18"/>
     </row>
-    <row r="44" spans="1:26" ht="57" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:26" ht="55.2">
       <c r="A44" s="18">
         <v>43</v>
       </c>
+      <c r="B44" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C44" t="s">
         <v>157</v>
       </c>
@@ -4404,10 +4530,13 @@
       </c>
       <c r="Z44" s="18"/>
     </row>
-    <row r="45" spans="1:26" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:26" ht="96.6">
       <c r="A45" s="18">
         <v>44</v>
       </c>
+      <c r="B45" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C45" t="s">
         <v>160</v>
       </c>
@@ -4461,10 +4590,13 @@
         <v>345</v>
       </c>
     </row>
-    <row r="46" spans="1:26" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:26" ht="69">
       <c r="A46" s="18">
         <v>45</v>
       </c>
+      <c r="B46" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C46" t="s">
         <v>164</v>
       </c>
@@ -4515,10 +4647,13 @@
       </c>
       <c r="Z46" s="18"/>
     </row>
-    <row r="47" spans="1:26" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:26" ht="69">
       <c r="A47" s="18">
         <v>46</v>
       </c>
+      <c r="B47" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C47" t="s">
         <v>170</v>
       </c>
@@ -4570,10 +4705,13 @@
       </c>
       <c r="Z47" s="18"/>
     </row>
-    <row r="48" spans="1:26" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:26" ht="124.2">
       <c r="A48" s="18">
         <v>47</v>
       </c>
+      <c r="B48" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C48" t="s">
         <v>173</v>
       </c>
@@ -4624,9 +4762,12 @@
       </c>
       <c r="Z48" s="18"/>
     </row>
-    <row r="49" spans="1:26" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:26" ht="207">
       <c r="A49" s="18">
         <v>48</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>294</v>
       </c>
       <c r="C49" t="s">
         <v>176</v>
@@ -4681,9 +4822,12 @@
         <v>358</v>
       </c>
     </row>
-    <row r="50" spans="1:26" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:26" ht="207">
       <c r="A50" s="18">
         <v>49</v>
+      </c>
+      <c r="B50" s="18" t="s">
+        <v>294</v>
       </c>
       <c r="C50" t="s">
         <v>180</v>
@@ -4738,10 +4882,13 @@
         <v>358</v>
       </c>
     </row>
-    <row r="51" spans="1:26" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:26" ht="82.8">
       <c r="A51" s="18">
         <v>50</v>
       </c>
+      <c r="B51" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C51" t="s">
         <v>183</v>
       </c>
@@ -4792,10 +4939,13 @@
       </c>
       <c r="Z51" s="18"/>
     </row>
-    <row r="52" spans="1:26" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:26" ht="82.8">
       <c r="A52" s="18">
         <v>51</v>
       </c>
+      <c r="B52" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C52" t="s">
         <v>187</v>
       </c>
@@ -4841,10 +4991,13 @@
       </c>
       <c r="Z52" s="18"/>
     </row>
-    <row r="53" spans="1:26" ht="270.75" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:26" ht="262.2">
       <c r="A53" s="18">
         <v>52</v>
       </c>
+      <c r="B53" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C53" t="s">
         <v>191</v>
       </c>
@@ -4895,10 +5048,13 @@
       </c>
       <c r="Z53" s="18"/>
     </row>
-    <row r="54" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:26" ht="27.6">
       <c r="A54" s="18">
         <v>53</v>
       </c>
+      <c r="B54" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C54" t="s">
         <v>193</v>
       </c>
@@ -4943,10 +5099,13 @@
       </c>
       <c r="Z54" s="18"/>
     </row>
-    <row r="55" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:26" ht="27.6">
       <c r="A55" s="18">
         <v>54</v>
       </c>
+      <c r="B55" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C55" t="s">
         <v>195</v>
       </c>
@@ -4992,10 +5151,13 @@
       </c>
       <c r="Z55" s="18"/>
     </row>
-    <row r="56" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:26" ht="27.6">
       <c r="A56" s="18">
         <v>55</v>
       </c>
+      <c r="B56" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C56" t="s">
         <v>197</v>
       </c>
@@ -5041,10 +5203,13 @@
       </c>
       <c r="Z56" s="18"/>
     </row>
-    <row r="57" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:26" ht="27.6">
       <c r="A57" s="18">
         <v>56</v>
       </c>
+      <c r="B57" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C57" t="s">
         <v>199</v>
       </c>
@@ -5089,10 +5254,13 @@
       </c>
       <c r="Z57" s="18"/>
     </row>
-    <row r="58" spans="1:26" ht="57" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:26" ht="55.2">
       <c r="A58" s="18">
         <v>57</v>
       </c>
+      <c r="B58" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C58" t="s">
         <v>201</v>
       </c>
@@ -5137,10 +5305,13 @@
       </c>
       <c r="Z58" s="18"/>
     </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:26">
       <c r="A59" s="18">
         <v>58</v>
       </c>
+      <c r="B59" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C59" t="s">
         <v>204</v>
       </c>
@@ -5182,10 +5353,13 @@
       </c>
       <c r="Z59" s="18"/>
     </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:26">
       <c r="A60" s="18">
         <v>59</v>
       </c>
+      <c r="B60" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C60" t="s">
         <v>206</v>
       </c>
@@ -5227,10 +5401,13 @@
       </c>
       <c r="Z60" s="18"/>
     </row>
-    <row r="61" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:26" ht="27.6">
       <c r="A61" s="18">
         <v>60</v>
       </c>
+      <c r="B61" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C61" t="s">
         <v>208</v>
       </c>
@@ -5272,10 +5449,13 @@
       </c>
       <c r="Z61" s="18"/>
     </row>
-    <row r="62" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:26" ht="27.6">
       <c r="A62" s="18">
         <v>61</v>
       </c>
+      <c r="B62" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C62" t="s">
         <v>210</v>
       </c>
@@ -5317,10 +5497,13 @@
       </c>
       <c r="Z62" s="18"/>
     </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:26">
       <c r="A63" s="18">
         <v>62</v>
       </c>
+      <c r="B63" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C63" t="s">
         <v>212</v>
       </c>
@@ -5363,10 +5546,13 @@
       </c>
       <c r="Z63" s="2"/>
     </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:26">
       <c r="A64" s="18">
         <v>63</v>
       </c>
+      <c r="B64" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C64" t="s">
         <v>214</v>
       </c>
@@ -5408,10 +5594,13 @@
       </c>
       <c r="Z64" s="18"/>
     </row>
-    <row r="65" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:26">
       <c r="A65" s="18">
         <v>64</v>
       </c>
+      <c r="B65" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C65" t="s">
         <v>216</v>
       </c>
@@ -5454,9 +5643,12 @@
       </c>
       <c r="Z65" s="18"/>
     </row>
-    <row r="66" spans="1:26" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:26" ht="96.6">
       <c r="A66" s="18">
         <v>65</v>
+      </c>
+      <c r="B66" s="18" t="s">
+        <v>294</v>
       </c>
       <c r="C66" t="s">
         <v>218</v>
@@ -5509,10 +5701,13 @@
       </c>
       <c r="Z66" s="2"/>
     </row>
-    <row r="67" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:26" ht="27.6">
       <c r="A67" s="18">
         <v>66</v>
       </c>
+      <c r="B67" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C67" t="s">
         <v>221</v>
       </c>
@@ -5558,10 +5753,13 @@
       </c>
       <c r="Z67" s="18"/>
     </row>
-    <row r="68" spans="1:26" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:26" ht="124.2">
       <c r="A68" s="18">
         <v>67</v>
       </c>
+      <c r="B68" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C68" t="s">
         <v>224</v>
       </c>
@@ -5606,10 +5804,13 @@
       </c>
       <c r="Z68" s="18"/>
     </row>
-    <row r="69" spans="1:26" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:26" ht="138">
       <c r="A69" s="18">
         <v>68</v>
       </c>
+      <c r="B69" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C69" t="s">
         <v>227</v>
       </c>
@@ -5660,10 +5861,13 @@
       </c>
       <c r="Z69" s="18"/>
     </row>
-    <row r="70" spans="1:26" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:26" ht="69">
       <c r="A70" s="18">
         <v>69</v>
       </c>
+      <c r="B70" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C70" t="s">
         <v>230</v>
       </c>
@@ -5708,10 +5912,13 @@
       </c>
       <c r="Z70" s="18"/>
     </row>
-    <row r="71" spans="1:26" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:26" ht="69">
       <c r="A71" s="18">
         <v>70</v>
       </c>
+      <c r="B71" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C71" t="s">
         <v>233</v>
       </c>
@@ -5756,10 +5963,13 @@
       </c>
       <c r="Z71" s="18"/>
     </row>
-    <row r="72" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:26" ht="27.6">
       <c r="A72" s="18">
         <v>71</v>
       </c>
+      <c r="B72" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C72" t="s">
         <v>235</v>
       </c>
@@ -5802,10 +6012,13 @@
       </c>
       <c r="Z72" s="18"/>
     </row>
-    <row r="73" spans="1:26" ht="216" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:26" ht="216" customHeight="1">
       <c r="A73" s="18">
         <v>72</v>
       </c>
+      <c r="B73" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C73" t="s">
         <v>237</v>
       </c>
@@ -5850,10 +6063,13 @@
       </c>
       <c r="Z73" s="18"/>
     </row>
-    <row r="74" spans="1:26" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:26" ht="41.4">
       <c r="A74" s="18">
         <v>73</v>
       </c>
+      <c r="B74" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C74" t="s">
         <v>241</v>
       </c>
@@ -5898,10 +6114,13 @@
       </c>
       <c r="Z74" s="18"/>
     </row>
-    <row r="75" spans="1:26" ht="57" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:26" ht="55.2">
       <c r="A75" s="18">
         <v>74</v>
       </c>
+      <c r="B75" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C75" t="s">
         <v>245</v>
       </c>
@@ -5946,10 +6165,13 @@
       </c>
       <c r="Z75" s="18"/>
     </row>
-    <row r="76" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:26" ht="27.6">
       <c r="A76" s="18">
         <v>75</v>
       </c>
+      <c r="B76" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C76" t="s">
         <v>249</v>
       </c>
@@ -5996,10 +6218,13 @@
       </c>
       <c r="Z76" s="2"/>
     </row>
-    <row r="77" spans="1:26" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:26" ht="138">
       <c r="A77" s="18">
         <v>76</v>
       </c>
+      <c r="B77" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C77" t="s">
         <v>252</v>
       </c>
@@ -6044,10 +6269,13 @@
       </c>
       <c r="Z77" s="18"/>
     </row>
-    <row r="78" spans="1:26" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:26" ht="41.4">
       <c r="A78" s="18">
         <v>77</v>
       </c>
+      <c r="B78" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C78" t="s">
         <v>256</v>
       </c>
@@ -6092,10 +6320,13 @@
       </c>
       <c r="Z78" s="18"/>
     </row>
-    <row r="79" spans="1:26" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:26" ht="82.8">
       <c r="A79" s="18">
         <v>78</v>
       </c>
+      <c r="B79" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C79" t="s">
         <v>260</v>
       </c>
@@ -6140,9 +6371,12 @@
       </c>
       <c r="Z79" s="18"/>
     </row>
-    <row r="80" spans="1:26" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:26" ht="409.5">
       <c r="A80" s="18">
         <v>79</v>
+      </c>
+      <c r="B80" s="18" t="s">
+        <v>294</v>
       </c>
       <c r="C80" t="s">
         <v>263</v>
@@ -6195,10 +6429,13 @@
       </c>
       <c r="Z80" s="2"/>
     </row>
-    <row r="81" spans="1:26" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:26" ht="96.6">
       <c r="A81" s="18">
         <v>80</v>
       </c>
+      <c r="B81" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C81" t="s">
         <v>266</v>
       </c>
@@ -6249,9 +6486,12 @@
       </c>
       <c r="Z81" s="18"/>
     </row>
-    <row r="82" spans="1:26" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:26" ht="409.5">
       <c r="A82" s="18">
         <v>81</v>
+      </c>
+      <c r="B82" s="18" t="s">
+        <v>294</v>
       </c>
       <c r="C82" t="s">
         <v>269</v>
@@ -6306,10 +6546,13 @@
         <v>384</v>
       </c>
     </row>
-    <row r="83" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:26" ht="27.6">
       <c r="A83" s="18">
         <v>82</v>
       </c>
+      <c r="B83" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C83" t="s">
         <v>272</v>
       </c>
@@ -6350,10 +6593,13 @@
         <v>17</v>
       </c>
     </row>
-    <row r="84" spans="1:26" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:26" ht="41.4">
       <c r="A84" s="18">
         <v>83</v>
       </c>
+      <c r="B84" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="C84" t="s">
         <v>275</v>
       </c>
@@ -6398,208 +6644,501 @@
         <v>17</v>
       </c>
     </row>
-    <row r="85" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:26">
+      <c r="B85" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="P85" s="18"/>
     </row>
-    <row r="86" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:26">
+      <c r="B86" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="P86" s="18"/>
     </row>
-    <row r="87" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:26">
+      <c r="B87" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
       <c r="K87" s="2"/>
       <c r="N87" s="5"/>
       <c r="P87" s="18"/>
     </row>
-    <row r="88" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:26">
+      <c r="B88" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="N88" s="8"/>
       <c r="P88" s="18"/>
     </row>
-    <row r="89" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:26">
+      <c r="B89" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I89" s="2"/>
       <c r="J89" s="2"/>
       <c r="K89" s="2"/>
     </row>
-    <row r="91" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:26">
+      <c r="B90" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="91" spans="1:26">
+      <c r="B91" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I91" s="2"/>
       <c r="J91" s="2"/>
       <c r="K91" s="2"/>
     </row>
-    <row r="95" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:26">
+      <c r="B92" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="93" spans="1:26">
+      <c r="B93" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="94" spans="1:26">
+      <c r="B94" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="95" spans="1:26">
+      <c r="B95" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
       <c r="K95" s="2"/>
       <c r="N95" s="5"/>
     </row>
-    <row r="96" spans="1:26" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:26">
+      <c r="B96" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I96" s="2"/>
       <c r="J96" s="2"/>
       <c r="K96" s="2"/>
       <c r="N96" s="5"/>
     </row>
-    <row r="97" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="97" spans="2:25">
+      <c r="B97" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
       <c r="K97" s="2"/>
     </row>
-    <row r="99" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="98" spans="2:25">
+      <c r="B98" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="99" spans="2:25">
+      <c r="B99" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I99" s="2"/>
       <c r="J99" s="2"/>
       <c r="K99" s="2"/>
       <c r="X99" s="9"/>
       <c r="Y99" s="9"/>
     </row>
-    <row r="101" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="100" spans="2:25">
+      <c r="B100" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="101" spans="2:25">
+      <c r="B101" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I101" s="2"/>
       <c r="J101" s="2"/>
       <c r="K101" s="2"/>
     </row>
-    <row r="102" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="102" spans="2:25">
+      <c r="B102" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="L102" s="2"/>
     </row>
-    <row r="103" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="103" spans="2:25">
+      <c r="B103" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="L103" s="2"/>
     </row>
-    <row r="104" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="104" spans="2:25">
+      <c r="B104" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I104" s="2"/>
       <c r="J104" s="2"/>
       <c r="K104" s="2"/>
       <c r="L104" s="2"/>
     </row>
-    <row r="111" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="105" spans="2:25">
+      <c r="B105" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="106" spans="2:25">
+      <c r="B106" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="107" spans="2:25">
+      <c r="B107" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="108" spans="2:25">
+      <c r="B108" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="109" spans="2:25">
+      <c r="B109" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="110" spans="2:25">
+      <c r="B110" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="111" spans="2:25">
+      <c r="B111" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I111" s="2"/>
       <c r="J111" s="2"/>
       <c r="K111" s="2"/>
     </row>
-    <row r="121" spans="9:11" x14ac:dyDescent="0.45">
+    <row r="112" spans="2:25">
+      <c r="B112" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="113" spans="2:11">
+      <c r="B113" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="114" spans="2:11">
+      <c r="B114" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="115" spans="2:11">
+      <c r="B115" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="116" spans="2:11">
+      <c r="B116" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="117" spans="2:11">
+      <c r="B117" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="118" spans="2:11">
+      <c r="B118" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="119" spans="2:11">
+      <c r="B119" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="120" spans="2:11">
+      <c r="B120" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="121" spans="2:11">
+      <c r="B121" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I121" s="2"/>
       <c r="J121" s="2"/>
       <c r="K121" s="2"/>
     </row>
-    <row r="123" spans="9:11" x14ac:dyDescent="0.45">
+    <row r="122" spans="2:11">
+      <c r="B122" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="123" spans="2:11">
+      <c r="B123" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I123" s="2"/>
       <c r="J123" s="2"/>
       <c r="K123" s="2"/>
     </row>
-    <row r="126" spans="9:11" x14ac:dyDescent="0.45">
+    <row r="124" spans="2:11">
+      <c r="B124" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="125" spans="2:11">
+      <c r="B125" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="126" spans="2:11">
+      <c r="B126" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I126" s="2"/>
       <c r="J126" s="2"/>
       <c r="K126" s="2"/>
     </row>
-    <row r="127" spans="9:11" x14ac:dyDescent="0.45">
+    <row r="127" spans="2:11">
+      <c r="B127" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I127" s="2"/>
       <c r="J127" s="2"/>
       <c r="K127" s="2"/>
     </row>
-    <row r="128" spans="9:11" x14ac:dyDescent="0.45">
+    <row r="128" spans="2:11">
+      <c r="B128" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I128" s="2"/>
       <c r="J128" s="2"/>
       <c r="K128" s="2"/>
     </row>
-    <row r="130" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="129" spans="2:14">
+      <c r="B129" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="130" spans="2:14">
+      <c r="B130" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I130" s="2"/>
       <c r="J130" s="2"/>
       <c r="K130" s="2"/>
       <c r="N130" s="5"/>
     </row>
-    <row r="131" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="131" spans="2:14">
+      <c r="B131" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I131" s="2"/>
       <c r="J131" s="2"/>
       <c r="K131" s="2"/>
     </row>
-    <row r="132" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="132" spans="2:14">
+      <c r="B132" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I132" s="2"/>
       <c r="J132" s="2"/>
       <c r="K132" s="2"/>
     </row>
-    <row r="133" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="133" spans="2:14">
+      <c r="B133" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I133" s="2"/>
       <c r="J133" s="2"/>
       <c r="K133" s="2"/>
     </row>
-    <row r="134" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="134" spans="2:14">
+      <c r="B134" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I134" s="2"/>
       <c r="J134" s="2"/>
       <c r="K134" s="2"/>
     </row>
-    <row r="135" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="135" spans="2:14">
+      <c r="B135" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I135" s="2"/>
       <c r="J135" s="2"/>
       <c r="K135" s="2"/>
     </row>
-    <row r="136" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="136" spans="2:14">
+      <c r="B136" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I136" s="2"/>
       <c r="J136" s="2"/>
       <c r="K136" s="2"/>
     </row>
-    <row r="137" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="137" spans="2:14">
+      <c r="B137" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I137" s="2"/>
       <c r="J137" s="2"/>
       <c r="K137" s="2"/>
     </row>
-    <row r="138" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="138" spans="2:14">
+      <c r="B138" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I138" s="2"/>
       <c r="J138" s="2"/>
       <c r="K138" s="2"/>
     </row>
-    <row r="139" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="139" spans="2:14">
+      <c r="B139" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I139" s="2"/>
       <c r="J139" s="2"/>
       <c r="K139" s="2"/>
     </row>
-    <row r="140" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="140" spans="2:14">
+      <c r="B140" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I140" s="2"/>
       <c r="J140" s="2"/>
       <c r="K140" s="2"/>
       <c r="N140" s="8"/>
     </row>
-    <row r="148" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="141" spans="2:14">
+      <c r="B141" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="142" spans="2:14">
+      <c r="B142" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="143" spans="2:14">
+      <c r="B143" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="144" spans="2:14">
+      <c r="B144" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="145" spans="2:25">
+      <c r="B145" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="146" spans="2:25">
+      <c r="B146" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="147" spans="2:25">
+      <c r="B147" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="148" spans="2:25">
+      <c r="B148" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I148" s="2"/>
       <c r="J148" s="2"/>
       <c r="K148" s="2"/>
       <c r="N148" s="8"/>
     </row>
-    <row r="150" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="149" spans="2:25">
+      <c r="B149" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="150" spans="2:25">
+      <c r="B150" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I150" s="2"/>
       <c r="J150" s="2"/>
       <c r="K150" s="2"/>
     </row>
-    <row r="151" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="151" spans="2:25">
+      <c r="B151" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I151" s="2"/>
       <c r="J151" s="2"/>
       <c r="K151" s="2"/>
     </row>
-    <row r="152" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="152" spans="2:25">
+      <c r="B152" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I152" s="2"/>
       <c r="J152" s="2"/>
       <c r="K152" s="2"/>
     </row>
-    <row r="153" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="153" spans="2:25">
+      <c r="B153" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I153" s="2"/>
       <c r="J153" s="2"/>
       <c r="K153" s="2"/>
     </row>
-    <row r="154" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="154" spans="2:25">
+      <c r="B154" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I154" s="2"/>
       <c r="J154" s="2"/>
       <c r="K154" s="2"/>
     </row>
-    <row r="155" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="155" spans="2:25">
+      <c r="B155" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I155" s="2"/>
       <c r="J155" s="2"/>
       <c r="K155" s="2"/>
     </row>
-    <row r="156" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="156" spans="2:25">
+      <c r="B156" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I156" s="2"/>
       <c r="J156" s="2"/>
       <c r="K156" s="2"/>
     </row>
-    <row r="157" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="157" spans="2:25">
+      <c r="B157" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I157" s="2"/>
       <c r="J157" s="2"/>
       <c r="K157" s="2"/>
     </row>
-    <row r="159" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="158" spans="2:25">
+      <c r="B158" s="18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="159" spans="2:25">
+      <c r="B159" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I159" s="2"/>
       <c r="J159" s="2"/>
       <c r="K159" s="2"/>
@@ -6607,35 +7146,50 @@
       <c r="X159" s="9"/>
       <c r="Y159" s="9"/>
     </row>
-    <row r="160" spans="9:25" x14ac:dyDescent="0.45">
+    <row r="160" spans="2:25">
+      <c r="B160" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I160" s="2"/>
       <c r="J160" s="2"/>
       <c r="K160" s="2"/>
       <c r="N160" s="5"/>
     </row>
-    <row r="161" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="161" spans="2:14">
+      <c r="B161" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I161" s="2"/>
       <c r="J161" s="2"/>
       <c r="K161" s="2"/>
     </row>
-    <row r="162" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="162" spans="2:14">
+      <c r="B162" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I162" s="2"/>
       <c r="J162" s="2"/>
       <c r="K162" s="2"/>
     </row>
-    <row r="163" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="163" spans="2:14">
+      <c r="B163" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I163" s="2"/>
       <c r="J163" s="2"/>
       <c r="K163" s="2"/>
     </row>
-    <row r="164" spans="9:14" x14ac:dyDescent="0.45">
+    <row r="164" spans="2:14">
+      <c r="B164" s="18" t="s">
+        <v>294</v>
+      </c>
       <c r="I164" s="2"/>
       <c r="J164" s="2"/>
       <c r="K164" s="2"/>
       <c r="N164" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y166" xr:uid="{A617E81B-AA39-4B57-8286-9F6F09A3BC0B}"/>
+  <autoFilter ref="A1:Y166"/>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test correct harmonized dataset column
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NHATS.xlsx
+++ b/baseline/data_processing_elements-NHATS.xlsx
@@ -2145,7 +2145,7 @@
     <col min="26" max="26" width="22.47265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="1" customFormat="1" ht="15.75">
+    <row r="1" spans="1:26" s="1" customFormat="1" ht="15.6">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -2225,7 +2225,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="15.75">
+    <row r="2" spans="1:26" ht="15.6">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="Z2" s="4"/>
     </row>
-    <row r="3" spans="1:26" s="21" customFormat="1" ht="42.75">
+    <row r="3" spans="1:26" s="21" customFormat="1" ht="41.4">
       <c r="A3" s="18">
         <v>2</v>
       </c>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="Z3" s="24"/>
     </row>
-    <row r="4" spans="1:26" ht="85.5">
+    <row r="4" spans="1:26" ht="82.8">
       <c r="A4" s="18">
         <v>3</v>
       </c>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="Z4" s="18"/>
     </row>
-    <row r="5" spans="1:26" ht="42.75">
+    <row r="5" spans="1:26" ht="41.4">
       <c r="A5" s="18">
         <v>4</v>
       </c>
@@ -2459,7 +2459,7 @@
       </c>
       <c r="Z5" s="18"/>
     </row>
-    <row r="6" spans="1:26" ht="99.75">
+    <row r="6" spans="1:26" ht="96.6">
       <c r="A6" s="18">
         <v>5</v>
       </c>
@@ -2571,7 +2571,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="28.5">
+    <row r="8" spans="1:26" ht="27.6">
       <c r="A8" s="18">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
addition of correct id_creation alogrithm
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NHATS.xlsx
+++ b/baseline/data_processing_elements-NHATS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17bc974f5891b333/Documents/ProPASS/Harmo/NHATS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="473" documentId="8_{9B09118A-A407-4BA8-95FA-BC26F1D8B61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBA1508C-6660-4CFE-B126-2D6410A279B3}"/>
+  <xr:revisionPtr revIDLastSave="476" documentId="8_{9B09118A-A407-4BA8-95FA-BC26F1D8B61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51597032-B74C-4090-A40D-D43252A6177A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F744FAC3-0BAB-4C7A-92B3-0824573F48DB}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1232" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1232" uniqueCount="398">
   <si>
     <t>index</t>
   </si>
@@ -1608,6 +1608,9 @@
   </si>
   <si>
     <t>input_keywords</t>
+  </si>
+  <si>
+    <t>id_creation</t>
   </si>
 </sst>
 </file>
@@ -2127,6 +2130,7 @@
     <col min="4" max="4" width="37.140625" customWidth="1"/>
     <col min="5" max="5" width="22.42578125" style="2" customWidth="1"/>
     <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="7" max="7" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="25.28515625" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
     <col min="11" max="11" width="57.42578125" style="2" customWidth="1"/>
@@ -2268,10 +2272,10 @@
         <v>27</v>
       </c>
       <c r="W2" s="4" t="s">
-        <v>28</v>
+        <v>397</v>
       </c>
       <c r="X2" s="4" t="s">
-        <v>28</v>
+        <v>287</v>
       </c>
       <c r="Y2" s="4"/>
     </row>

</xml_diff>

<commit_message>
corrected alogrithms from before/after report
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NHATS.xlsx
+++ b/baseline/data_processing_elements-NHATS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17bc974f5891b333/Documents/ProPASS/Harmo/NHATS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="476" documentId="8_{9B09118A-A407-4BA8-95FA-BC26F1D8B61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51597032-B74C-4090-A40D-D43252A6177A}"/>
+  <xr:revisionPtr revIDLastSave="516" documentId="8_{9B09118A-A407-4BA8-95FA-BC26F1D8B61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2B3F1E4-ED23-46FD-B870-2A8246C190EA}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F744FAC3-0BAB-4C7A-92B3-0824573F48DB}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F744FAC3-0BAB-4C7A-92B3-0824573F48DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1232" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1234" uniqueCount="400">
   <si>
     <t>index</t>
   </si>
@@ -1055,9 +1055,6 @@
     <t>hrs/week</t>
   </si>
   <si>
-    <t>recode (3 = 1; c(1,2) = 0; c(-9,-8,-7,-1) = NA; ELSE = NA)</t>
-  </si>
-  <si>
     <t>hh11dmarstat</t>
   </si>
   <si>
@@ -1077,9 +1074,6 @@
 </t>
   </si>
   <si>
-    <t>recode (c(1,2) = 1; c(3,4,5,6) = 0; c(-9,-8,-7) = NA; -1 = NA; ELSE = NA)</t>
-  </si>
-  <si>
     <t>“Living with a partner” does not imply ever married. Since this category cannot be classified with certainty into the DataSchema categories, the variable is considered incompatible.</t>
   </si>
   <si>
@@ -1194,9 +1188,6 @@
 3 = Good;
 4 = Fair;
 5 = Poor</t>
-  </si>
-  <si>
-    <t>recode (5 = 1; 4 = 2; 3 = 3; c(1,2) = 4; ELSE = NA)</t>
   </si>
   <si>
     <t>hc11disescn1; hc11disescn2</t>
@@ -1227,9 +1218,6 @@
 )</t>
   </si>
   <si>
-    <t>the study does not include an “other” category, therefor "No" category cannot be produced.</t>
-  </si>
-  <si>
     <t>hc11disescn4; hc11disescn5</t>
   </si>
   <si>
@@ -1273,25 +1261,6 @@
 R11 HC3 SP HAD KIDNEY CANCER;
 R11 HC3 SP HAD OTHER CANCER;
 R11 HC3 SP HAD SKIN CANCER</t>
-  </si>
-  <si>
-    <t>case_when(
-hc11cancerty2 %in% c(1,7) | 
-hc11cancerty3 %in% c(1,7) | 
-hc11cancerty4 %in% c(1,7) | 
-hc11cancerty5 %in% c(1,7) | 
-hc11cancerty6 %in% c(1,7) | 
-hc11cancerty7 %in% c(1,7) | 
-hc11cancerty8 %in% c(1,7) ~ 1;
-hc11cancerty2 == 2 &amp; 
-hc11cancerty3 == 2 &amp; 
-hc11cancerty4 == 2 &amp; 
-hc11cancerty5 == 2 &amp; 
-hc11cancerty6 == 2 &amp; 
-hc11cancerty7 == 2 &amp; 
-hc11cancerty8 == 2 ~ 0;
-TRUE ~ NA_integer
-)</t>
   </si>
   <si>
     <t>hc11disescn9</t>
@@ -1343,20 +1312,6 @@
 1 = YES;
 2 = NO
 </t>
-  </si>
-  <si>
-    <t>case_when(
-hc11trbfalbck %in% c(1,2,3) | hc11aslep30mn %in% c(1,2,3) ~ 1;
-hc11trbfalbck %in% c(4,7) &amp; hc11aslep30mn %in% c(4,5) ~ 0;
-TRUE ~ NA_integer
-)</t>
-  </si>
-  <si>
-    <t>case_when(
-dt11getoplcs1 == 1 | ha11howgtstr7 == 1 ~ 1;
-dt11getoplcs1 == 2 &amp; ha11howgtstr7 == 2 ~ 0;
-TRUE ~ NA_integer
-)</t>
   </si>
   <si>
     <t>case_when(
@@ -1570,47 +1525,96 @@
 )</t>
   </si>
   <si>
+    <t>R11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Questionnaire </t>
+  </si>
+  <si>
+    <t>JSN Comment/Question</t>
+  </si>
+  <si>
+    <t>dataschema_variable_label</t>
+  </si>
+  <si>
+    <t>unit/other_format</t>
+  </si>
+  <si>
+    <t>Categories::label</t>
+  </si>
+  <si>
+    <t>categories/format</t>
+  </si>
+  <si>
+    <t>field_type</t>
+  </si>
+  <si>
+    <t>input_keywords</t>
+  </si>
+  <si>
+    <t>id_creation</t>
+  </si>
+  <si>
+    <t>lf11doccup</t>
+  </si>
+  <si>
+    <t>R11 D CURRENT OCCUPATION CATEGORY</t>
+  </si>
+  <si>
+    <t>recode (3 = 1; 1:2= 0; -7:-9 = NA;  -1=NA; ELSE = NA)</t>
+  </si>
+  <si>
+    <t>recode (1:2= 1; 3:6 = 0; -7:-9 = NA; -1 = NA; ELSE = NA)</t>
+  </si>
+  <si>
+    <t>recode (5=1; 4=2; 3=3; 1:2=4; ELSE = NA)</t>
+  </si>
+  <si>
+    <t>case_when(
+hc11cancerty2 %in% c(1,7) | 
+hc11cancerty3 %in% c(1,7) | 
+hc11cancerty4 %in% c(1,7) | 
+hc11cancerty5 %in% c(1,7) | 
+hc11cancerty6 %in% c(1,7) | 
+hc11cancerty7 %in% c(1,7) | 
+hc11cancerty8 %in% c(1,7) ~ 1;
+hc11cancerty2 == 2 &amp; 
+hc11cancerty3 == 2 &amp; 
+hc11cancerty4 == 2 &amp; 
+hc11cancerty5 == 2 &amp; 
+hc11cancerty6 == 2 &amp; 
+hc11cancerty7 == 2 &amp; 
+hc11cancerty8 == 2 ~ 0;
+TRUE ~ NA_integer_
+)</t>
+  </si>
+  <si>
+    <t>case_when(
+hc11trbfalbck %in% c(1,2,3) | hc11aslep30mn %in% c(1,2,3) ~ 1;
+hc11trbfalbck %in% c(4,7) &amp; hc11aslep30mn %in% c(4,5) ~ 0;
+TRUE ~ NA_integer_
+)</t>
+  </si>
+  <si>
+    <t>case_when(
+dt11getoplcs1 == 1 | ha11howgtstr7 == 1 ~ 1;
+dt11getoplcs1 == 2 &amp; ha11howgtstr7 == 2 ~ 0;
+TRUE ~ NA_integer_
+)</t>
+  </si>
+  <si>
     <t>case_when(
   hw11howtallft %in% c(-7, -8, -9, -1) |
-  hw11howtallin %in% c(-7, -8, -9, -1) |
-  hw11currweigh %in% c(-7, -8, -9, -1) ~ NA_real_,
-  !is.na(hw11howtallft) &amp; !is.na(hw11howtallin) &amp; !is.na(hw11currweigh) ~ {
-    height_m &lt;- ((hw11howtallft * 12) + hw11howtallin) * 0.0254
-    weight_kg &lt;- hw11currweigh * 0.453592
-    weight_kg / (height_m^2)
-  },
+    hw11howtallin %in% c(-7, -8, -9, -1) |
+    hw11currweigh %in% c(-7, -8, -9, -1) ~ NA_real_,
+  !is.na(hw11howtallft) &amp; !is.na(hw11howtallin) &amp; !is.na(hw11currweigh) ~
+    (hw11currweigh * 0.453592) /
+    ((((hw11howtallft * 12) + hw11howtallin) * 0.0254)^2),
   TRUE ~ NA_real_
 )</t>
   </si>
   <si>
-    <t>R11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Questionnaire </t>
-  </si>
-  <si>
-    <t>JSN Comment/Question</t>
-  </si>
-  <si>
-    <t>dataschema_variable_label</t>
-  </si>
-  <si>
-    <t>unit/other_format</t>
-  </si>
-  <si>
-    <t>Categories::label</t>
-  </si>
-  <si>
-    <t>categories/format</t>
-  </si>
-  <si>
-    <t>field_type</t>
-  </si>
-  <si>
-    <t>input_keywords</t>
-  </si>
-  <si>
-    <t>id_creation</t>
+    <t>the study does not include an “other” category, therefore "No" category cannot be produced.</t>
   </si>
 </sst>
 </file>
@@ -2122,32 +2126,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC73F24-28B6-451D-9DE2-0CD6B57BA63C}">
   <dimension ref="A1:Y164"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1"/>
-    <col min="2" max="2" width="24.28515625" customWidth="1"/>
+    <col min="1" max="1" width="9.1328125" customWidth="1"/>
+    <col min="2" max="2" width="24.265625" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="37.140625" customWidth="1"/>
-    <col min="5" max="5" width="22.42578125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="25.28515625" customWidth="1"/>
+    <col min="4" max="4" width="37.1328125" customWidth="1"/>
+    <col min="5" max="5" width="22.3984375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.1328125" customWidth="1"/>
+    <col min="7" max="7" width="24.1328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="25.265625" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
-    <col min="11" max="11" width="57.42578125" style="2" customWidth="1"/>
-    <col min="12" max="12" width="70.42578125" style="3" customWidth="1"/>
-    <col min="13" max="15" width="22.140625" customWidth="1"/>
-    <col min="16" max="16" width="24.5703125" customWidth="1"/>
-    <col min="17" max="18" width="22.140625" customWidth="1"/>
-    <col min="19" max="19" width="31.85546875" customWidth="1"/>
-    <col min="20" max="20" width="21.140625" customWidth="1"/>
-    <col min="21" max="21" width="28.42578125" customWidth="1"/>
-    <col min="22" max="22" width="23.7109375" customWidth="1"/>
-    <col min="23" max="23" width="27.7109375" customWidth="1"/>
-    <col min="24" max="24" width="61.5703125" customWidth="1"/>
-    <col min="25" max="25" width="22.42578125" customWidth="1"/>
+    <col min="11" max="11" width="57.3984375" style="2" customWidth="1"/>
+    <col min="12" max="12" width="70.3984375" style="3" customWidth="1"/>
+    <col min="13" max="15" width="22.1328125" customWidth="1"/>
+    <col min="16" max="16" width="24.59765625" customWidth="1"/>
+    <col min="17" max="18" width="22.1328125" customWidth="1"/>
+    <col min="19" max="19" width="31.86328125" customWidth="1"/>
+    <col min="20" max="20" width="21.1328125" customWidth="1"/>
+    <col min="21" max="21" width="28.3984375" customWidth="1"/>
+    <col min="22" max="22" width="23.73046875" customWidth="1"/>
+    <col min="23" max="23" width="27.73046875" customWidth="1"/>
+    <col min="24" max="24" width="61.59765625" customWidth="1"/>
+    <col min="25" max="25" width="22.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -2158,7 +2162,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>3</v>
@@ -2167,10 +2171,10 @@
         <v>4</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="I1" s="10" t="s">
         <v>1</v>
@@ -2182,10 +2186,10 @@
         <v>278</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="N1" s="15" t="s">
         <v>280</v>
@@ -2200,7 +2204,7 @@
         <v>283</v>
       </c>
       <c r="R1" s="10" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="S1" s="16" t="s">
         <v>9</v>
@@ -2221,10 +2225,10 @@
         <v>8</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2256,11 +2260,11 @@
         <v>16</v>
       </c>
       <c r="N2" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="O2" s="11"/>
       <c r="P2" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="Q2" s="11"/>
       <c r="R2" s="11"/>
@@ -2272,14 +2276,14 @@
         <v>27</v>
       </c>
       <c r="W2" s="4" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
       <c r="X2" s="4" t="s">
         <v>287</v>
       </c>
       <c r="Y2" s="4"/>
     </row>
-    <row r="3" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2306,18 +2310,18 @@
         <v>286</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>384</v>
+        <v>377</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="L3" s="5"/>
       <c r="N3" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="O3" s="13"/>
       <c r="P3" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="Q3" s="13"/>
       <c r="R3" s="13"/>
@@ -2336,7 +2340,7 @@
       </c>
       <c r="Y3" s="4"/>
     </row>
-    <row r="4" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2371,11 +2375,11 @@
         <v>291</v>
       </c>
       <c r="N4" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="O4" s="11"/>
       <c r="P4" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="Q4" s="11"/>
       <c r="R4" s="11"/>
@@ -2392,7 +2396,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2429,10 +2433,10 @@
         <v>32</v>
       </c>
       <c r="N5" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U5" s="4" t="s">
         <v>26</v>
@@ -2447,7 +2451,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="120" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2477,10 +2481,10 @@
       </c>
       <c r="L6" s="5"/>
       <c r="N6" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P6" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="S6" s="2"/>
       <c r="U6" t="s">
@@ -2499,7 +2503,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="225" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2531,10 +2535,10 @@
         <v>297</v>
       </c>
       <c r="N7" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P7" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="S7" s="2"/>
       <c r="U7" t="s">
@@ -2553,7 +2557,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2588,10 +2592,10 @@
         <v>305</v>
       </c>
       <c r="N8" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P8" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U8" t="s">
         <v>26</v>
@@ -2606,7 +2610,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2632,19 +2636,19 @@
         <v>286</v>
       </c>
       <c r="J9" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="K9" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="N9" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P9" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U9" s="4" t="s">
         <v>26</v>
@@ -2656,10 +2660,10 @@
         <v>51</v>
       </c>
       <c r="X9" s="12" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2687,14 +2691,14 @@
       <c r="K10" t="s">
         <v>308</v>
       </c>
-      <c r="M10" t="s">
+      <c r="N10" t="s">
+        <v>380</v>
+      </c>
+      <c r="P10" t="s">
+        <v>381</v>
+      </c>
+      <c r="R10" t="s">
         <v>309</v>
-      </c>
-      <c r="N10" t="s">
-        <v>388</v>
-      </c>
-      <c r="P10" t="s">
-        <v>389</v>
       </c>
       <c r="U10" t="s">
         <v>26</v>
@@ -2709,7 +2713,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2732,28 +2736,34 @@
         <v>286</v>
       </c>
       <c r="J11" t="s">
-        <v>306</v>
+        <v>390</v>
+      </c>
+      <c r="K11" t="s">
+        <v>391</v>
+      </c>
+      <c r="M11" t="s">
+        <v>13</v>
       </c>
       <c r="N11" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P11" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U11" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="V11" t="s">
-        <v>300</v>
+        <v>27</v>
       </c>
       <c r="W11" t="s">
-        <v>14</v>
-      </c>
-      <c r="X11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="X11" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2784,14 +2794,14 @@
       <c r="K12" t="s">
         <v>304</v>
       </c>
-      <c r="L12" t="s">
+      <c r="L12" s="5" t="s">
         <v>305</v>
       </c>
       <c r="N12" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P12" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U12" t="s">
         <v>26</v>
@@ -2803,10 +2813,11 @@
         <v>38</v>
       </c>
       <c r="X12" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25" ht="180" x14ac:dyDescent="0.25">
+        <v>392</v>
+      </c>
+      <c r="Y12" s="2"/>
+    </row>
+    <row r="13" spans="1:25" ht="171" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2832,19 +2843,19 @@
         <v>286</v>
       </c>
       <c r="J13" t="s">
+        <v>310</v>
+      </c>
+      <c r="K13" t="s">
         <v>311</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="L13" s="5" t="s">
-        <v>313</v>
-      </c>
       <c r="N13" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P13" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U13" t="s">
         <v>14</v>
@@ -2858,11 +2869,11 @@
       <c r="X13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="Y13" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="14" spans="1:25" ht="180" x14ac:dyDescent="0.25">
+      <c r="Y13" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" ht="171" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2888,19 +2899,19 @@
         <v>286</v>
       </c>
       <c r="J14" t="s">
+        <v>310</v>
+      </c>
+      <c r="K14" t="s">
         <v>311</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="L14" s="5" t="s">
-        <v>313</v>
-      </c>
       <c r="N14" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P14" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U14" t="s">
         <v>26</v>
@@ -2912,10 +2923,11 @@
         <v>38</v>
       </c>
       <c r="X14" s="2" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+        <v>393</v>
+      </c>
+      <c r="Y14" s="2"/>
+    </row>
+    <row r="15" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2944,10 +2956,10 @@
         <v>306</v>
       </c>
       <c r="N15" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P15" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U15" s="4" t="s">
         <v>14</v>
@@ -2962,7 +2974,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="135" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2989,22 +3001,22 @@
         <v>286</v>
       </c>
       <c r="J16" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="M16" t="s">
         <v>316</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="L16" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="M16" t="s">
-        <v>318</v>
-      </c>
       <c r="N16" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P16" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U16" t="s">
         <v>26</v>
@@ -3016,10 +3028,10 @@
         <v>75</v>
       </c>
       <c r="X16" s="2" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="17" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3048,10 +3060,10 @@
         <v>306</v>
       </c>
       <c r="N17" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P17" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U17" s="4" t="s">
         <v>26</v>
@@ -3060,13 +3072,13 @@
         <v>27</v>
       </c>
       <c r="W17" s="4" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="X17" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3093,19 +3105,19 @@
         <v>286</v>
       </c>
       <c r="J18" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="K18" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="M18" t="s">
         <v>82</v>
       </c>
       <c r="N18" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P18" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U18" t="s">
         <v>26</v>
@@ -3117,10 +3129,10 @@
         <v>75</v>
       </c>
       <c r="X18" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="19" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3149,10 +3161,10 @@
         <v>306</v>
       </c>
       <c r="N19" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P19" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U19" s="4" t="s">
         <v>26</v>
@@ -3161,13 +3173,13 @@
         <v>27</v>
       </c>
       <c r="W19" s="4" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="X19" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:24" ht="210" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3193,19 +3205,19 @@
         <v>286</v>
       </c>
       <c r="J20" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="M20" t="s">
         <v>324</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="M20" t="s">
-        <v>326</v>
-      </c>
       <c r="N20" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P20" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U20" t="s">
         <v>26</v>
@@ -3217,10 +3229,10 @@
         <v>75</v>
       </c>
       <c r="X20" s="2" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3247,19 +3259,19 @@
         <v>286</v>
       </c>
       <c r="J21" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="K21" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="M21" t="s">
         <v>74</v>
       </c>
       <c r="N21" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P21" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U21" t="s">
         <v>26</v>
@@ -3271,10 +3283,10 @@
         <v>75</v>
       </c>
       <c r="X21" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="22" spans="1:24" ht="60" x14ac:dyDescent="0.25">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" ht="57" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3300,19 +3312,19 @@
         <v>286</v>
       </c>
       <c r="J22" t="s">
+        <v>328</v>
+      </c>
+      <c r="K22" t="s">
+        <v>329</v>
+      </c>
+      <c r="L22" s="5" t="s">
         <v>330</v>
       </c>
-      <c r="K22" t="s">
-        <v>331</v>
-      </c>
-      <c r="L22" s="5" t="s">
-        <v>332</v>
-      </c>
       <c r="N22" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P22" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U22" t="s">
         <v>26</v>
@@ -3324,10 +3336,10 @@
         <v>38</v>
       </c>
       <c r="X22" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3356,13 +3368,13 @@
         <v>306</v>
       </c>
       <c r="N23" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P23" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="24" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>23</v>
       </c>
@@ -3388,10 +3400,10 @@
         <v>306</v>
       </c>
       <c r="N24" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P24" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U24" s="4" t="s">
         <v>14</v>
@@ -3406,7 +3418,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>24</v>
       </c>
@@ -3435,10 +3447,10 @@
         <v>306</v>
       </c>
       <c r="N25" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P25" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U25" s="4" t="s">
         <v>14</v>
@@ -3453,7 +3465,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3482,10 +3494,10 @@
         <v>306</v>
       </c>
       <c r="N26" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P26" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U26" s="4" t="s">
         <v>14</v>
@@ -3500,7 +3512,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>26</v>
       </c>
@@ -3529,10 +3541,10 @@
         <v>306</v>
       </c>
       <c r="N27" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P27" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U27" s="4" t="s">
         <v>14</v>
@@ -3547,7 +3559,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3577,10 +3589,10 @@
         <v>306</v>
       </c>
       <c r="N28" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P28" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U28" s="4" t="s">
         <v>14</v>
@@ -3595,7 +3607,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3624,10 +3636,10 @@
         <v>306</v>
       </c>
       <c r="N29" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P29" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U29" s="4" t="s">
         <v>14</v>
@@ -3642,7 +3654,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3671,10 +3683,10 @@
         <v>306</v>
       </c>
       <c r="N30" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P30" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U30" s="4" t="s">
         <v>14</v>
@@ -3689,7 +3701,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:24" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3718,10 +3730,10 @@
         <v>306</v>
       </c>
       <c r="N31" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P31" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U31" s="4" t="s">
         <v>14</v>
@@ -3736,7 +3748,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3765,10 +3777,10 @@
         <v>306</v>
       </c>
       <c r="N32" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P32" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U32" s="4" t="s">
         <v>14</v>
@@ -3783,7 +3795,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3812,10 +3824,10 @@
         <v>306</v>
       </c>
       <c r="N33" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P33" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U33" s="4" t="s">
         <v>14</v>
@@ -3830,7 +3842,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3859,10 +3871,10 @@
         <v>306</v>
       </c>
       <c r="N34" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P34" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U34" s="4" t="s">
         <v>14</v>
@@ -3877,7 +3889,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3906,10 +3918,10 @@
         <v>306</v>
       </c>
       <c r="N35" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P35" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U35" s="4" t="s">
         <v>14</v>
@@ -3924,7 +3936,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3953,10 +3965,10 @@
         <v>306</v>
       </c>
       <c r="N36" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P36" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U36" s="4" t="s">
         <v>14</v>
@@ -3971,7 +3983,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A37">
         <v>36</v>
       </c>
@@ -4000,10 +4012,10 @@
         <v>306</v>
       </c>
       <c r="N37" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P37" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U37" s="4" t="s">
         <v>14</v>
@@ -4018,7 +4030,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>37</v>
       </c>
@@ -4048,10 +4060,10 @@
         <v>306</v>
       </c>
       <c r="N38" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P38" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U38" s="4" t="s">
         <v>14</v>
@@ -4066,7 +4078,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="1:25" s="2" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:25" s="2" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39">
         <v>38</v>
       </c>
@@ -4097,11 +4109,11 @@
       <c r="L39" s="3"/>
       <c r="M39"/>
       <c r="N39" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="O39"/>
       <c r="P39" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="Q39"/>
       <c r="R39"/>
@@ -4119,7 +4131,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="40" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A40">
         <v>39</v>
       </c>
@@ -4149,10 +4161,10 @@
         <v>306</v>
       </c>
       <c r="N40" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P40" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U40" s="4" t="s">
         <v>14</v>
@@ -4167,7 +4179,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:25" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A41">
         <v>40</v>
       </c>
@@ -4196,10 +4208,10 @@
         <v>306</v>
       </c>
       <c r="N41" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P41" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U41" s="4" t="s">
         <v>14</v>
@@ -4214,7 +4226,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A42">
         <v>41</v>
       </c>
@@ -4243,10 +4255,10 @@
         <v>306</v>
       </c>
       <c r="N42" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P42" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U42" s="4" t="s">
         <v>14</v>
@@ -4261,7 +4273,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A43">
         <v>42</v>
       </c>
@@ -4291,10 +4303,10 @@
         <v>306</v>
       </c>
       <c r="N43" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P43" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U43" s="4" t="s">
         <v>14</v>
@@ -4309,7 +4321,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:25" ht="57" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>43</v>
       </c>
@@ -4338,10 +4350,10 @@
         <v>306</v>
       </c>
       <c r="N44" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P44" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U44" s="4" t="s">
         <v>14</v>
@@ -4356,7 +4368,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:25" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A45">
         <v>44</v>
       </c>
@@ -4382,26 +4394,26 @@
         <v>286</v>
       </c>
       <c r="J45" t="s">
+        <v>332</v>
+      </c>
+      <c r="K45" t="s">
+        <v>333</v>
+      </c>
+      <c r="L45" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="K45" t="s">
-        <v>335</v>
-      </c>
-      <c r="L45" s="5" t="s">
-        <v>336</v>
-      </c>
       <c r="N45" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P45" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="S45" s="2"/>
       <c r="U45" t="s">
         <v>14</v>
       </c>
       <c r="V45" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="W45" s="4" t="s">
         <v>14</v>
@@ -4410,10 +4422,10 @@
         <v>14</v>
       </c>
       <c r="Y45" s="2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="46" spans="1:25" ht="75" x14ac:dyDescent="0.25">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="46" spans="1:25" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A46">
         <v>45</v>
       </c>
@@ -4439,7 +4451,7 @@
         <v>286</v>
       </c>
       <c r="J46" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="K46" s="2" t="s">
         <v>164</v>
@@ -4448,16 +4460,16 @@
         <v>165</v>
       </c>
       <c r="N46" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P46" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U46" t="s">
         <v>14</v>
       </c>
       <c r="V46" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="W46" s="2" t="s">
         <v>14</v>
@@ -4466,7 +4478,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:25" ht="75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:25" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A47">
         <v>46</v>
       </c>
@@ -4493,19 +4505,19 @@
         <v>286</v>
       </c>
       <c r="J47" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="K47" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="L47" s="5" t="s">
         <v>165</v>
       </c>
       <c r="N47" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P47" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U47" t="s">
         <v>26</v>
@@ -4517,10 +4529,10 @@
         <v>51</v>
       </c>
       <c r="X47" s="2" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="48" spans="1:25" ht="135" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="48" spans="1:25" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4546,19 +4558,19 @@
         <v>286</v>
       </c>
       <c r="J48" t="s">
+        <v>340</v>
+      </c>
+      <c r="K48" t="s">
+        <v>341</v>
+      </c>
+      <c r="L48" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="K48" t="s">
-        <v>343</v>
-      </c>
-      <c r="L48" s="5" t="s">
-        <v>344</v>
-      </c>
       <c r="N48" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P48" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U48" t="s">
         <v>26</v>
@@ -4570,10 +4582,10 @@
         <v>38</v>
       </c>
       <c r="X48" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="49" spans="1:25" ht="225" x14ac:dyDescent="0.25">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="49" spans="1:25" ht="213.75" x14ac:dyDescent="0.45">
       <c r="A49">
         <v>48</v>
       </c>
@@ -4599,19 +4611,19 @@
         <v>286</v>
       </c>
       <c r="J49" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="N49" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P49" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="S49" s="2"/>
       <c r="U49" t="s">
@@ -4624,13 +4636,13 @@
         <v>51</v>
       </c>
       <c r="X49" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="Y49" s="2" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="50" spans="1:25" ht="225" x14ac:dyDescent="0.25">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="50" spans="1:25" ht="213.75" x14ac:dyDescent="0.45">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4656,19 +4668,19 @@
         <v>286</v>
       </c>
       <c r="J50" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="N50" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P50" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="S50" s="2"/>
       <c r="U50" t="s">
@@ -4681,13 +4693,13 @@
         <v>51</v>
       </c>
       <c r="X50" s="2" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="Y50" s="2" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="51" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="51" spans="1:25" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4713,19 +4725,19 @@
         <v>286</v>
       </c>
       <c r="J51" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="K51" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="L51" s="5" t="s">
         <v>182</v>
       </c>
       <c r="N51" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P51" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U51" t="s">
         <v>26</v>
@@ -4737,10 +4749,10 @@
         <v>51</v>
       </c>
       <c r="X51" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="52" spans="1:25" ht="120" x14ac:dyDescent="0.25">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="52" spans="1:25" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4770,10 +4782,10 @@
       </c>
       <c r="L52" s="5"/>
       <c r="N52" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P52" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U52" s="4" t="s">
         <v>14</v>
@@ -4788,7 +4800,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:25" ht="285" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:25" ht="270.75" x14ac:dyDescent="0.45">
       <c r="A53">
         <v>52</v>
       </c>
@@ -4814,19 +4826,19 @@
         <v>286</v>
       </c>
       <c r="J53" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="L53" s="5" t="s">
         <v>357</v>
       </c>
-      <c r="K53" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="L53" s="5" t="s">
-        <v>362</v>
-      </c>
       <c r="N53" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P53" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U53" t="s">
         <v>26</v>
@@ -4838,10 +4850,10 @@
         <v>51</v>
       </c>
       <c r="X53" s="2" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="54" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="54" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A54">
         <v>53</v>
       </c>
@@ -4870,10 +4882,10 @@
         <v>306</v>
       </c>
       <c r="N54" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P54" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U54" s="4" t="s">
         <v>14</v>
@@ -4888,7 +4900,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="55" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A55">
         <v>54</v>
       </c>
@@ -4918,10 +4930,10 @@
       </c>
       <c r="L55" s="5"/>
       <c r="N55" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P55" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U55" s="4" t="s">
         <v>14</v>
@@ -4936,7 +4948,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="56" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A56">
         <v>55</v>
       </c>
@@ -4966,10 +4978,10 @@
       </c>
       <c r="L56" s="5"/>
       <c r="N56" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P56" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U56" s="4" t="s">
         <v>14</v>
@@ -4984,7 +4996,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A57">
         <v>56</v>
       </c>
@@ -5013,10 +5025,10 @@
         <v>306</v>
       </c>
       <c r="N57" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P57" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U57" s="4" t="s">
         <v>14</v>
@@ -5031,7 +5043,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:25" ht="57" x14ac:dyDescent="0.45">
       <c r="A58">
         <v>57</v>
       </c>
@@ -5060,10 +5072,10 @@
         <v>306</v>
       </c>
       <c r="N58" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P58" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U58" s="4" t="s">
         <v>14</v>
@@ -5078,7 +5090,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="59" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A59">
         <v>58</v>
       </c>
@@ -5104,10 +5116,10 @@
         <v>306</v>
       </c>
       <c r="N59" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P59" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U59" s="4" t="s">
         <v>14</v>
@@ -5122,7 +5134,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A60">
         <v>59</v>
       </c>
@@ -5148,10 +5160,10 @@
         <v>306</v>
       </c>
       <c r="N60" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P60" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U60" s="4" t="s">
         <v>14</v>
@@ -5166,7 +5178,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A61">
         <v>60</v>
       </c>
@@ -5192,10 +5204,10 @@
         <v>306</v>
       </c>
       <c r="N61" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P61" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U61" s="4" t="s">
         <v>14</v>
@@ -5210,7 +5222,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="62" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A62">
         <v>61</v>
       </c>
@@ -5236,10 +5248,10 @@
         <v>306</v>
       </c>
       <c r="N62" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P62" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U62" s="4" t="s">
         <v>14</v>
@@ -5254,7 +5266,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="63" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A63">
         <v>62</v>
       </c>
@@ -5280,10 +5292,10 @@
         <v>306</v>
       </c>
       <c r="N63" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P63" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="S63" s="2"/>
       <c r="U63" s="4" t="s">
@@ -5300,7 +5312,7 @@
       </c>
       <c r="Y63" s="2"/>
     </row>
-    <row r="64" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A64">
         <v>63</v>
       </c>
@@ -5326,10 +5338,10 @@
         <v>306</v>
       </c>
       <c r="N64" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P64" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U64" s="4" t="s">
         <v>14</v>
@@ -5344,7 +5356,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="65" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A65">
         <v>64</v>
       </c>
@@ -5371,10 +5383,10 @@
         <v>306</v>
       </c>
       <c r="N65" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P65" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U65" s="4" t="s">
         <v>14</v>
@@ -5389,7 +5401,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:25" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A66">
         <v>65</v>
       </c>
@@ -5415,19 +5427,19 @@
         <v>286</v>
       </c>
       <c r="J66" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="K66" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="L66" s="5" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="N66" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P66" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="S66" s="2"/>
       <c r="U66" t="s">
@@ -5440,11 +5452,11 @@
         <v>38</v>
       </c>
       <c r="X66" s="2" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="Y66" s="2"/>
     </row>
-    <row r="67" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A67">
         <v>66</v>
       </c>
@@ -5474,10 +5486,10 @@
         <v>306</v>
       </c>
       <c r="N67" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P67" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U67" s="4" t="s">
         <v>14</v>
@@ -5492,7 +5504,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="68" spans="1:25" ht="135" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:25" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A68">
         <v>67</v>
       </c>
@@ -5521,10 +5533,10 @@
         <v>306</v>
       </c>
       <c r="N68" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P68" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U68" s="4" t="s">
         <v>14</v>
@@ -5539,7 +5551,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="69" spans="1:25" ht="150" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:25" ht="142.5" x14ac:dyDescent="0.45">
       <c r="A69">
         <v>68</v>
       </c>
@@ -5565,19 +5577,19 @@
         <v>286</v>
       </c>
       <c r="J69" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="L69" s="5" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="N69" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P69" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U69" t="s">
         <v>26</v>
@@ -5589,10 +5601,10 @@
         <v>51</v>
       </c>
       <c r="X69" s="2" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="70" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="70" spans="1:25" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A70">
         <v>69</v>
       </c>
@@ -5621,10 +5633,10 @@
         <v>306</v>
       </c>
       <c r="N70" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P70" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U70" s="4" t="s">
         <v>14</v>
@@ -5639,7 +5651,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="71" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:25" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A71">
         <v>70</v>
       </c>
@@ -5668,10 +5680,10 @@
         <v>306</v>
       </c>
       <c r="N71" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P71" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U71" s="4" t="s">
         <v>14</v>
@@ -5686,7 +5698,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="72" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A72">
         <v>71</v>
       </c>
@@ -5713,10 +5725,10 @@
         <v>306</v>
       </c>
       <c r="N72" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P72" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U72" s="4" t="s">
         <v>14</v>
@@ -5731,7 +5743,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="73" spans="1:25" ht="216" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:25" ht="216" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73">
         <v>72</v>
       </c>
@@ -5760,10 +5772,10 @@
         <v>306</v>
       </c>
       <c r="N73" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P73" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U73" s="4" t="s">
         <v>14</v>
@@ -5778,7 +5790,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="74" spans="1:25" ht="75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:25" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A74">
         <v>73</v>
       </c>
@@ -5807,10 +5819,10 @@
         <v>306</v>
       </c>
       <c r="N74" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P74" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U74" s="4" t="s">
         <v>14</v>
@@ -5825,7 +5837,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="1:25" ht="75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:25" ht="57" x14ac:dyDescent="0.45">
       <c r="A75">
         <v>74</v>
       </c>
@@ -5854,10 +5866,10 @@
         <v>306</v>
       </c>
       <c r="N75" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P75" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U75" s="4" t="s">
         <v>14</v>
@@ -5872,7 +5884,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="76" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A76">
         <v>75</v>
       </c>
@@ -5902,10 +5914,10 @@
         <v>306</v>
       </c>
       <c r="N76" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P76" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="S76" s="2"/>
       <c r="U76" s="4" t="s">
@@ -5922,7 +5934,7 @@
       </c>
       <c r="Y76" s="2"/>
     </row>
-    <row r="77" spans="1:25" ht="165" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:25" ht="142.5" x14ac:dyDescent="0.45">
       <c r="A77">
         <v>76</v>
       </c>
@@ -5951,10 +5963,10 @@
         <v>306</v>
       </c>
       <c r="N77" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P77" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U77" s="4" t="s">
         <v>14</v>
@@ -5969,7 +5981,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:25" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A78">
         <v>77</v>
       </c>
@@ -5998,10 +6010,10 @@
         <v>306</v>
       </c>
       <c r="N78" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P78" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U78" s="4" t="s">
         <v>14</v>
@@ -6016,7 +6028,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="79" spans="1:25" ht="120" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:25" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A79">
         <v>78</v>
       </c>
@@ -6045,10 +6057,10 @@
         <v>306</v>
       </c>
       <c r="N79" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P79" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U79" s="4" t="s">
         <v>14</v>
@@ -6063,7 +6075,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:25" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:25" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A80">
         <v>79</v>
       </c>
@@ -6089,19 +6101,19 @@
         <v>286</v>
       </c>
       <c r="J80" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="K80" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="L80" s="5" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="N80" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P80" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="S80" s="2"/>
       <c r="U80" t="s">
@@ -6114,11 +6126,11 @@
         <v>51</v>
       </c>
       <c r="X80" s="2" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="Y80" s="2"/>
     </row>
-    <row r="81" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:25" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A81">
         <v>80</v>
       </c>
@@ -6144,19 +6156,19 @@
         <v>286</v>
       </c>
       <c r="J81" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="K81" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="L81" s="5" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="N81" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P81" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U81" t="s">
         <v>26</v>
@@ -6168,10 +6180,10 @@
         <v>51</v>
       </c>
       <c r="X81" s="2" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="82" spans="1:25" ht="409.5" x14ac:dyDescent="0.25">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="82" spans="1:25" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A82">
         <v>81</v>
       </c>
@@ -6197,19 +6209,19 @@
         <v>286</v>
       </c>
       <c r="J82" s="6" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="K82" s="2" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="L82" s="5" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="N82" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P82" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="S82" s="2"/>
       <c r="U82" t="s">
@@ -6222,13 +6234,13 @@
         <v>51</v>
       </c>
       <c r="X82" s="2" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="Y82" s="2" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="83" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="83" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A83">
         <v>82</v>
       </c>
@@ -6254,10 +6266,10 @@
         <v>306</v>
       </c>
       <c r="N83" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P83" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U83" s="4" t="s">
         <v>14</v>
@@ -6272,7 +6284,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="84" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:25" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A84">
         <v>83</v>
       </c>
@@ -6302,10 +6314,10 @@
       </c>
       <c r="L84" s="5"/>
       <c r="N84" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="P84" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="U84" s="4" t="s">
         <v>14</v>
@@ -6320,189 +6332,189 @@
         <v>14</v>
       </c>
     </row>
-    <row r="87" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:25" x14ac:dyDescent="0.45">
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
       <c r="L87" s="5"/>
     </row>
-    <row r="88" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:25" x14ac:dyDescent="0.45">
       <c r="L88" s="8"/>
     </row>
-    <row r="89" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:25" x14ac:dyDescent="0.45">
       <c r="H89" s="2"/>
       <c r="I89" s="2"/>
     </row>
-    <row r="91" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:25" x14ac:dyDescent="0.45">
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
     </row>
-    <row r="95" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:25" x14ac:dyDescent="0.45">
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
       <c r="L95" s="5"/>
     </row>
-    <row r="96" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:25" x14ac:dyDescent="0.45">
       <c r="H96" s="2"/>
       <c r="I96" s="2"/>
       <c r="L96" s="5"/>
     </row>
-    <row r="97" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="97" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
     </row>
-    <row r="99" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="99" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>
       <c r="W99" s="9"/>
       <c r="X99" s="9"/>
     </row>
-    <row r="101" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="101" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H101" s="2"/>
       <c r="I101" s="2"/>
     </row>
-    <row r="102" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="102" spans="8:24" x14ac:dyDescent="0.45">
       <c r="J102" s="2"/>
     </row>
-    <row r="103" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="103" spans="8:24" x14ac:dyDescent="0.45">
       <c r="J103" s="2"/>
     </row>
-    <row r="104" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="104" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H104" s="2"/>
       <c r="I104" s="2"/>
       <c r="J104" s="2"/>
     </row>
-    <row r="111" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="111" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H111" s="2"/>
       <c r="I111" s="2"/>
     </row>
-    <row r="121" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="121" spans="8:9" x14ac:dyDescent="0.45">
       <c r="H121" s="2"/>
       <c r="I121" s="2"/>
     </row>
-    <row r="123" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="123" spans="8:9" x14ac:dyDescent="0.45">
       <c r="H123" s="2"/>
       <c r="I123" s="2"/>
     </row>
-    <row r="126" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="126" spans="8:9" x14ac:dyDescent="0.45">
       <c r="H126" s="2"/>
       <c r="I126" s="2"/>
     </row>
-    <row r="127" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="127" spans="8:9" x14ac:dyDescent="0.45">
       <c r="H127" s="2"/>
       <c r="I127" s="2"/>
     </row>
-    <row r="128" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="128" spans="8:9" x14ac:dyDescent="0.45">
       <c r="H128" s="2"/>
       <c r="I128" s="2"/>
     </row>
-    <row r="130" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H130" s="2"/>
       <c r="I130" s="2"/>
       <c r="L130" s="5"/>
     </row>
-    <row r="131" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H131" s="2"/>
       <c r="I131" s="2"/>
     </row>
-    <row r="132" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H132" s="2"/>
       <c r="I132" s="2"/>
     </row>
-    <row r="133" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H133" s="2"/>
       <c r="I133" s="2"/>
     </row>
-    <row r="134" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H134" s="2"/>
       <c r="I134" s="2"/>
     </row>
-    <row r="135" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H135" s="2"/>
       <c r="I135" s="2"/>
     </row>
-    <row r="136" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H136" s="2"/>
       <c r="I136" s="2"/>
     </row>
-    <row r="137" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H137" s="2"/>
       <c r="I137" s="2"/>
     </row>
-    <row r="138" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H138" s="2"/>
       <c r="I138" s="2"/>
     </row>
-    <row r="139" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H139" s="2"/>
       <c r="I139" s="2"/>
     </row>
-    <row r="140" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H140" s="2"/>
       <c r="I140" s="2"/>
       <c r="L140" s="8"/>
     </row>
-    <row r="148" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="148" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H148" s="2"/>
       <c r="I148" s="2"/>
       <c r="L148" s="8"/>
     </row>
-    <row r="150" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="150" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H150" s="2"/>
       <c r="I150" s="2"/>
     </row>
-    <row r="151" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="151" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H151" s="2"/>
       <c r="I151" s="2"/>
     </row>
-    <row r="152" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="152" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H152" s="2"/>
       <c r="I152" s="2"/>
     </row>
-    <row r="153" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="153" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H153" s="2"/>
       <c r="I153" s="2"/>
     </row>
-    <row r="154" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="154" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H154" s="2"/>
       <c r="I154" s="2"/>
     </row>
-    <row r="155" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="155" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H155" s="2"/>
       <c r="I155" s="2"/>
     </row>
-    <row r="156" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="156" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H156" s="2"/>
       <c r="I156" s="2"/>
     </row>
-    <row r="157" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="157" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H157" s="2"/>
       <c r="I157" s="2"/>
     </row>
-    <row r="159" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="159" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H159" s="2"/>
       <c r="I159" s="2"/>
       <c r="L159" s="5"/>
       <c r="W159" s="9"/>
       <c r="X159" s="9"/>
     </row>
-    <row r="160" spans="8:24" x14ac:dyDescent="0.25">
+    <row r="160" spans="8:24" x14ac:dyDescent="0.45">
       <c r="H160" s="2"/>
       <c r="I160" s="2"/>
       <c r="L160" s="5"/>
     </row>
-    <row r="161" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="161" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H161" s="2"/>
       <c r="I161" s="2"/>
     </row>
-    <row r="162" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="162" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H162" s="2"/>
       <c r="I162" s="2"/>
     </row>
-    <row r="163" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="163" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H163" s="2"/>
       <c r="I163" s="2"/>
     </row>
-    <row r="164" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="164" spans="8:12" x14ac:dyDescent="0.45">
       <c r="H164" s="2"/>
       <c r="I164" s="2"/>
       <c r="L164" s="5"/>

</xml_diff>